<commit_message>
close review of serialisation
</commit_message>
<xml_diff>
--- a/tests/data/alphabet_vocab.xlsx
+++ b/tests/data/alphabet_vocab.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="103">
   <si>
     <t xml:space="preserve">ConceptScheme</t>
   </si>
@@ -58,12 +58,21 @@
     <t xml:space="preserve">Narrower</t>
   </si>
   <si>
+    <t xml:space="preserve">RelatedScheme</t>
+  </si>
+  <si>
     <t xml:space="preserve">Related</t>
   </si>
   <si>
+    <t xml:space="preserve">CloseMatchScheme</t>
+  </si>
+  <si>
     <t xml:space="preserve">CloseMatch</t>
   </si>
   <si>
+    <t xml:space="preserve">ExactMatchScheme</t>
+  </si>
+  <si>
     <t xml:space="preserve">ExactMatch</t>
   </si>
   <si>
@@ -154,6 +163,9 @@
     <t xml:space="preserve">A house is a residential building typically split into different functional rooms. Houses can be built from a variety of materials and traditional houses will often reflect materials that are available locally.</t>
   </si>
   <si>
+    <t xml:space="preserve">Structure</t>
+  </si>
+  <si>
     <t xml:space="preserve">https://en.wikipedia.org/wiki/House</t>
   </si>
   <si>
@@ -220,7 +232,7 @@
     <t xml:space="preserve">Octopus</t>
   </si>
   <si>
-    <t xml:space="preserve">An octopus is a soft-bodied, eight-limbed mollusc of the class Cephalopod. They live in the ocean and are known for their intelligence, and in some species ability to camoflage and expell ink when threatened.</t>
+    <t xml:space="preserve">An octopus is a soft-bodied, eight-limbed mollusc of the class Cephalopod. They live in the ocean and are known for their intelligence, and in some species have the ability to camoflage and expell ink when threatened.</t>
   </si>
   <si>
     <t xml:space="preserve">https://en.wikipedia.org/wiki/Octopus</t>
@@ -369,7 +381,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -379,7 +391,19 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFF5429"/>
+        <bgColor rgb="FFFF860D"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF860D"/>
         <bgColor rgb="FFFF8080"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFD428"/>
+        <bgColor rgb="FFFFFF00"/>
       </patternFill>
     </fill>
   </fills>
@@ -417,7 +441,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -436,6 +460,14 @@
     </xf>
     <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
@@ -504,8 +536,8 @@
       <rgbColor rgb="FF3366FF"/>
       <rgbColor rgb="FF33CCCC"/>
       <rgbColor rgb="FF99CC00"/>
-      <rgbColor rgb="FFFFCC00"/>
-      <rgbColor rgb="FFFF9900"/>
+      <rgbColor rgb="FFFFD428"/>
+      <rgbColor rgb="FFFF860D"/>
       <rgbColor rgb="FFFF5429"/>
       <rgbColor rgb="FF666699"/>
       <rgbColor rgb="FF969696"/>
@@ -633,7 +665,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:P27"/>
+  <dimension ref="A1:S27"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="22.86"/>
@@ -648,12 +680,14 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="2" width="11.85"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="11.85"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="13.25"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="13" style="1" width="9.46"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="18.08"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="1" width="30.88"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="18.26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="18.68"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="22.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="16" style="1" width="16.69"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="1" width="30.88"/>
   </cols>
   <sheetData>
-    <row r="1" s="5" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" s="7" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -690,692 +724,713 @@
       <c r="L1" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="3" t="s">
+      <c r="M1" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="3" t="s">
+      <c r="N1" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="3" t="s">
+      <c r="O1" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="3" t="s">
+      <c r="P1" s="6" t="s">
         <v>15</v>
+      </c>
+      <c r="Q1" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="R1" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="S1" s="3" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="I2" s="6" t="s">
-        <v>20</v>
+        <v>22</v>
+      </c>
+      <c r="I2" s="8" t="s">
+        <v>23</v>
       </c>
       <c r="L2" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="P2" s="7" t="s">
-        <v>22</v>
+        <v>24</v>
+      </c>
+      <c r="S2" s="9" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="I3" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="I3" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="L3" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="L3" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="P3" s="7" t="s">
-        <v>25</v>
+      <c r="S3" s="9" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="L4" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="P4" s="7" t="s">
-        <v>29</v>
+        <v>31</v>
+      </c>
+      <c r="S4" s="9" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="I5" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="L5" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="L5" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="P5" s="7" t="s">
-        <v>32</v>
+      <c r="S5" s="9" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="L6" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="P6" s="7" t="s">
-        <v>35</v>
+        <v>31</v>
+      </c>
+      <c r="S6" s="9" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="L7" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="P7" s="7" t="s">
-        <v>38</v>
+        <v>31</v>
+      </c>
+      <c r="S7" s="9" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="L8" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="P8" s="7" t="s">
-        <v>41</v>
+        <v>31</v>
+      </c>
+      <c r="S8" s="9" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="P9" s="7" t="s">
-        <v>44</v>
+        <v>46</v>
+      </c>
+      <c r="L9" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="S9" s="9" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="P10" s="7" t="s">
-        <v>47</v>
+        <v>50</v>
+      </c>
+      <c r="S10" s="9" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="P11" s="7" t="s">
-        <v>50</v>
+        <v>53</v>
+      </c>
+      <c r="S11" s="9" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="L12" s="1" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="M12" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="P12" s="7" t="s">
-        <v>55</v>
+        <v>19</v>
+      </c>
+      <c r="N12" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="S12" s="9" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="L13" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="P13" s="7" t="s">
-        <v>58</v>
+        <v>24</v>
+      </c>
+      <c r="S13" s="9" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="L14" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="P14" s="7" t="s">
-        <v>61</v>
+        <v>31</v>
+      </c>
+      <c r="S14" s="9" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="I15" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="P15" s="7" t="s">
-        <v>64</v>
+        <v>67</v>
+      </c>
+      <c r="L15" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="S15" s="9" t="s">
+        <v>68</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="I16" s="2" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="L16" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="P16" s="7" t="s">
-        <v>67</v>
+        <v>31</v>
+      </c>
+      <c r="S16" s="9" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="I17" s="2" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="L17" s="1" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="I18" s="2" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="L18" s="1" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="M18" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="P18" s="7" t="s">
-        <v>71</v>
+        <v>19</v>
+      </c>
+      <c r="N18" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="S18" s="9" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="I19" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="P19" s="7" t="s">
-        <v>74</v>
+        <v>77</v>
+      </c>
+      <c r="S19" s="9" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="I20" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="P20" s="7" t="s">
-        <v>77</v>
+        <v>80</v>
+      </c>
+      <c r="S20" s="9" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="I21" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="P21" s="7" t="s">
-        <v>80</v>
+        <v>83</v>
+      </c>
+      <c r="S21" s="9" t="s">
+        <v>84</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="I22" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="P22" s="7" t="s">
-        <v>83</v>
+        <v>86</v>
+      </c>
+      <c r="S22" s="9" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="I23" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="P23" s="7" t="s">
-        <v>86</v>
+        <v>89</v>
+      </c>
+      <c r="S23" s="9" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="I24" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="P24" s="7" t="s">
-        <v>89</v>
+        <v>92</v>
+      </c>
+      <c r="S24" s="9" t="s">
+        <v>93</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="I25" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="P25" s="7" t="s">
-        <v>92</v>
+        <v>95</v>
+      </c>
+      <c r="S25" s="9" t="s">
+        <v>96</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="I26" s="2" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="L26" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="P26" s="7" t="s">
-        <v>95</v>
+        <v>31</v>
+      </c>
+      <c r="S26" s="9" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="I27" s="2" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="L27" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="P27" s="7" t="s">
-        <v>98</v>
+        <v>31</v>
+      </c>
+      <c r="S27" s="9" t="s">
+        <v>102</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="P2" r:id="rId1" display="https://en.wikipedia.org/wiki/Apple"/>
-    <hyperlink ref="P3" r:id="rId2" display="https://en.wikipedia.org/wiki/Banana"/>
-    <hyperlink ref="P4" r:id="rId3" display="https://en.wikipedia.org/wiki/Cat"/>
-    <hyperlink ref="P5" r:id="rId4" display="https://en.wikipedia.org/wiki/Dog"/>
-    <hyperlink ref="P6" r:id="rId5" display="https://en.wikipedia.org/wiki/Elephant"/>
-    <hyperlink ref="P7" r:id="rId6" display="https://en.wikipedia.org/wiki/Fox"/>
-    <hyperlink ref="P8" r:id="rId7" display="https://en.wikipedia.org/wiki/Goat"/>
-    <hyperlink ref="P9" r:id="rId8" display="https://en.wikipedia.org/wiki/House"/>
-    <hyperlink ref="P10" r:id="rId9" display="https://en.wikipedia.org/wiki/Imagination"/>
-    <hyperlink ref="P11" r:id="rId10" display="https://en.wikipedia.org/wiki/Jungle"/>
-    <hyperlink ref="P12" r:id="rId11" display="https://en.wikipedia.org/wiki/King"/>
-    <hyperlink ref="P13" r:id="rId12" display="https://en.wikipedia.org/wiki/Lemon"/>
-    <hyperlink ref="P14" r:id="rId13" display="https://en.wikipedia.org/wiki/Mouse"/>
-    <hyperlink ref="P15" r:id="rId14" display="https://en.wikipedia.org/wiki/Nest"/>
-    <hyperlink ref="P16" r:id="rId15" display="https://en.wikipedia.org/wiki/Octopus"/>
-    <hyperlink ref="P18" r:id="rId16" display="https://en.wikipedia.org/wiki/Queen_regnant"/>
-    <hyperlink ref="P19" r:id="rId17" display="https://en.wikipedia.org/wiki/Rain"/>
-    <hyperlink ref="P20" r:id="rId18" display="https://en.wikipedia.org/wiki/Sun"/>
-    <hyperlink ref="P21" r:id="rId19" display="https://en.wikipedia.org/wiki/Train"/>
-    <hyperlink ref="P22" r:id="rId20" display="https://en.wikipedia.org/wiki/Umbrella"/>
-    <hyperlink ref="P23" r:id="rId21" display="https://en.wikipedia.org/wiki/Village"/>
-    <hyperlink ref="P24" r:id="rId22" display="https://en.wikipedia.org/wiki/Wheel"/>
-    <hyperlink ref="P25" r:id="rId23" display="https://en.wikipedia.org/wiki/Xylophone"/>
-    <hyperlink ref="P26" r:id="rId24" display="https://en.wikipedia.org/wiki/Yak"/>
-    <hyperlink ref="P27" r:id="rId25" display="https://en.wikipedia.org/wiki/Zebra"/>
+    <hyperlink ref="S2" r:id="rId1" display="https://en.wikipedia.org/wiki/Apple"/>
+    <hyperlink ref="S3" r:id="rId2" display="https://en.wikipedia.org/wiki/Banana"/>
+    <hyperlink ref="S4" r:id="rId3" display="https://en.wikipedia.org/wiki/Cat"/>
+    <hyperlink ref="S5" r:id="rId4" display="https://en.wikipedia.org/wiki/Dog"/>
+    <hyperlink ref="S6" r:id="rId5" display="https://en.wikipedia.org/wiki/Elephant"/>
+    <hyperlink ref="S7" r:id="rId6" display="https://en.wikipedia.org/wiki/Fox"/>
+    <hyperlink ref="S8" r:id="rId7" display="https://en.wikipedia.org/wiki/Goat"/>
+    <hyperlink ref="S9" r:id="rId8" display="https://en.wikipedia.org/wiki/House"/>
+    <hyperlink ref="S10" r:id="rId9" display="https://en.wikipedia.org/wiki/Imagination"/>
+    <hyperlink ref="S11" r:id="rId10" display="https://en.wikipedia.org/wiki/Jungle"/>
+    <hyperlink ref="S12" r:id="rId11" display="https://en.wikipedia.org/wiki/King"/>
+    <hyperlink ref="S13" r:id="rId12" display="https://en.wikipedia.org/wiki/Lemon"/>
+    <hyperlink ref="S14" r:id="rId13" display="https://en.wikipedia.org/wiki/Mouse"/>
+    <hyperlink ref="S15" r:id="rId14" display="https://en.wikipedia.org/wiki/Nest"/>
+    <hyperlink ref="S16" r:id="rId15" display="https://en.wikipedia.org/wiki/Octopus"/>
+    <hyperlink ref="S18" r:id="rId16" display="https://en.wikipedia.org/wiki/Queen_regnant"/>
+    <hyperlink ref="S19" r:id="rId17" display="https://en.wikipedia.org/wiki/Rain"/>
+    <hyperlink ref="S20" r:id="rId18" display="https://en.wikipedia.org/wiki/Sun"/>
+    <hyperlink ref="S21" r:id="rId19" display="https://en.wikipedia.org/wiki/Train"/>
+    <hyperlink ref="S22" r:id="rId20" display="https://en.wikipedia.org/wiki/Umbrella"/>
+    <hyperlink ref="S23" r:id="rId21" display="https://en.wikipedia.org/wiki/Village"/>
+    <hyperlink ref="S24" r:id="rId22" display="https://en.wikipedia.org/wiki/Wheel"/>
+    <hyperlink ref="S25" r:id="rId23" display="https://en.wikipedia.org/wiki/Xylophone"/>
+    <hyperlink ref="S26" r:id="rId24" display="https://en.wikipedia.org/wiki/Yak"/>
+    <hyperlink ref="S27" r:id="rId25" display="https://en.wikipedia.org/wiki/Zebra"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>

</xml_diff>

<commit_message>
tests and sample vocabulary alignment
</commit_message>
<xml_diff>
--- a/tests/data/alphabet_vocab.xlsx
+++ b/tests/data/alphabet_vocab.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="260" uniqueCount="114">
   <si>
     <t xml:space="preserve">ConceptScheme</t>
   </si>
@@ -244,6 +244,9 @@
     <t xml:space="preserve">A parrot is a bird with a strong curved beak, upright stance and clawed feet. They are broadly classified into four familes and are found in the wild, and sometimes as pets. They are among the most intelligent of birds and typically eat seeds, nuts or fruit.</t>
   </si>
   <si>
+    <t xml:space="preserve">https://en.wikipedia.org/wiki/Parrot</t>
+  </si>
+  <si>
     <t xml:space="preserve">A queen is a female monarch, equivalent in rank, title and position to a King. She will reign over a realm known as a kingdom.</t>
   </si>
   <si>
@@ -274,6 +277,9 @@
     <t xml:space="preserve">A train typically describes a series of connected vehicles that run along a railway track. They can be used to transport people or freight. A train is typically pulled by a locomotive (engine) though some trains might have their propulsion distributed acrooss carriages and powered by an external power-source. </t>
   </si>
   <si>
+    <t xml:space="preserve">Artifact</t>
+  </si>
+  <si>
     <t xml:space="preserve">https://en.wikipedia.org/wiki/Train</t>
   </si>
   <si>
@@ -329,6 +335,33 @@
   </si>
   <si>
     <t xml:space="preserve">https://en.wikipedia.org/wiki/Zebra</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A multicellular, eukaryotic organism. Animals are different from other living things in that they cannot produce their own food, and tend to have to ingest organic material to survive.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://en.wikipedia.org/wiki/Animal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">An object or thing created as the result of human craftmanship.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">An often edible component of a plant or vegetable that hosts seeds.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://en.wikipedia.org/wiki/Fruit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A leadership role assigned to a person who rules over a kingdom or realm.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://en.wikipedia.org/wiki/Monarch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A physical arrangement of components that conforms to a template or pattern. Can be the result of natural or artificial processes.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://en.wikipedia.org/wiki/Structure</t>
   </si>
 </sst>
 </file>
@@ -338,7 +371,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -369,6 +402,13 @@
     </font>
     <font>
       <sz val="12"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF0000FF"/>
       <name val="Arial"/>
       <family val="2"/>
       <charset val="1"/>
@@ -441,7 +481,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -479,6 +519,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -665,7 +709,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:S27"/>
+  <dimension ref="A1:S32"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="22.86"/>
@@ -1158,6 +1202,9 @@
       <c r="L17" s="1" t="s">
         <v>31</v>
       </c>
+      <c r="S17" s="10" t="s">
+        <v>74</v>
+      </c>
     </row>
     <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
@@ -1176,7 +1223,7 @@
         <v>58</v>
       </c>
       <c r="I18" s="2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="L18" s="1" t="s">
         <v>57</v>
@@ -1188,7 +1235,7 @@
         <v>55</v>
       </c>
       <c r="S18" s="9" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1202,16 +1249,16 @@
         <v>21</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="I19" s="2" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="S19" s="9" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1225,16 +1272,16 @@
         <v>21</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="I20" s="2" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="S20" s="9" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1248,16 +1295,19 @@
         <v>21</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="I21" s="2" t="s">
-        <v>83</v>
+        <v>84</v>
+      </c>
+      <c r="L21" s="1" t="s">
+        <v>85</v>
       </c>
       <c r="S21" s="9" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1271,16 +1321,19 @@
         <v>21</v>
       </c>
       <c r="D22" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="F22" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="I22" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="L22" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="F22" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="I22" s="2" t="s">
-        <v>86</v>
-      </c>
       <c r="S22" s="9" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1294,16 +1347,16 @@
         <v>21</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="I23" s="2" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="S23" s="9" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1317,16 +1370,19 @@
         <v>21</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="I24" s="2" t="s">
-        <v>92</v>
+        <v>94</v>
+      </c>
+      <c r="L24" s="1" t="s">
+        <v>85</v>
       </c>
       <c r="S24" s="9" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1340,16 +1396,19 @@
         <v>21</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="I25" s="2" t="s">
-        <v>95</v>
+        <v>97</v>
+      </c>
+      <c r="L25" s="1" t="s">
+        <v>85</v>
       </c>
       <c r="S25" s="9" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1363,19 +1422,19 @@
         <v>21</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="I26" s="2" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="L26" s="1" t="s">
         <v>31</v>
       </c>
       <c r="S26" s="9" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1389,19 +1448,131 @@
         <v>21</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="I27" s="2" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="L27" s="1" t="s">
         <v>31</v>
       </c>
       <c r="S27" s="9" t="s">
-        <v>102</v>
+        <v>104</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="F28" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="I28" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="S28" s="10" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D29" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="F29" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="I29" s="2" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D30" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="F30" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="I30" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="S30" s="10" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D31" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="F31" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="I31" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="S31" s="10" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D32" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="F32" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="I32" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="S32" s="10" t="s">
+        <v>113</v>
       </c>
     </row>
   </sheetData>
@@ -1421,16 +1592,21 @@
     <hyperlink ref="S14" r:id="rId13" display="https://en.wikipedia.org/wiki/Mouse"/>
     <hyperlink ref="S15" r:id="rId14" display="https://en.wikipedia.org/wiki/Nest"/>
     <hyperlink ref="S16" r:id="rId15" display="https://en.wikipedia.org/wiki/Octopus"/>
-    <hyperlink ref="S18" r:id="rId16" display="https://en.wikipedia.org/wiki/Queen_regnant"/>
-    <hyperlink ref="S19" r:id="rId17" display="https://en.wikipedia.org/wiki/Rain"/>
-    <hyperlink ref="S20" r:id="rId18" display="https://en.wikipedia.org/wiki/Sun"/>
-    <hyperlink ref="S21" r:id="rId19" display="https://en.wikipedia.org/wiki/Train"/>
-    <hyperlink ref="S22" r:id="rId20" display="https://en.wikipedia.org/wiki/Umbrella"/>
-    <hyperlink ref="S23" r:id="rId21" display="https://en.wikipedia.org/wiki/Village"/>
-    <hyperlink ref="S24" r:id="rId22" display="https://en.wikipedia.org/wiki/Wheel"/>
-    <hyperlink ref="S25" r:id="rId23" display="https://en.wikipedia.org/wiki/Xylophone"/>
-    <hyperlink ref="S26" r:id="rId24" display="https://en.wikipedia.org/wiki/Yak"/>
-    <hyperlink ref="S27" r:id="rId25" display="https://en.wikipedia.org/wiki/Zebra"/>
+    <hyperlink ref="S17" r:id="rId16" display="https://en.wikipedia.org/wiki/Parrot"/>
+    <hyperlink ref="S18" r:id="rId17" display="https://en.wikipedia.org/wiki/Queen_regnant"/>
+    <hyperlink ref="S19" r:id="rId18" display="https://en.wikipedia.org/wiki/Rain"/>
+    <hyperlink ref="S20" r:id="rId19" display="https://en.wikipedia.org/wiki/Sun"/>
+    <hyperlink ref="S21" r:id="rId20" display="https://en.wikipedia.org/wiki/Train"/>
+    <hyperlink ref="S22" r:id="rId21" display="https://en.wikipedia.org/wiki/Umbrella"/>
+    <hyperlink ref="S23" r:id="rId22" display="https://en.wikipedia.org/wiki/Village"/>
+    <hyperlink ref="S24" r:id="rId23" display="https://en.wikipedia.org/wiki/Wheel"/>
+    <hyperlink ref="S25" r:id="rId24" display="https://en.wikipedia.org/wiki/Xylophone"/>
+    <hyperlink ref="S26" r:id="rId25" display="https://en.wikipedia.org/wiki/Yak"/>
+    <hyperlink ref="S27" r:id="rId26" display="https://en.wikipedia.org/wiki/Zebra"/>
+    <hyperlink ref="S28" r:id="rId27" display="https://en.wikipedia.org/wiki/Animal"/>
+    <hyperlink ref="S30" r:id="rId28" display="https://en.wikipedia.org/wiki/Fruit"/>
+    <hyperlink ref="S31" r:id="rId29" display="https://en.wikipedia.org/wiki/Monarch"/>
+    <hyperlink ref="S32" r:id="rId30" display="https://en.wikipedia.org/wiki/Structure"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>

</xml_diff>

<commit_message>
serialisation improvements and tests
</commit_message>
<xml_diff>
--- a/tests/data/alphabet_vocab.xlsx
+++ b/tests/data/alphabet_vocab.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="260" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="266" uniqueCount="116">
   <si>
     <t xml:space="preserve">ConceptScheme</t>
   </si>
@@ -103,7 +103,7 @@
     <t xml:space="preserve">Banana</t>
   </si>
   <si>
-    <t xml:space="preserve">A banana is an elongated, edible fruit (botalically a berry) of herbaceous plants of the genus Musa.</t>
+    <t xml:space="preserve">A banana is an elongated, edible fruit (botanically a berry) of herbaceous plants of the genus Musa.</t>
   </si>
   <si>
     <t xml:space="preserve">https://en.wikipedia.org/wiki/Banana</t>
@@ -362,6 +362,12 @@
   </si>
   <si>
     <t xml:space="preserve">https://en.wikipedia.org/wiki/Structure</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test.TestAlphabetVocab</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A duplicated definition which, if assigned to kgmeta:Description, ought to be identified as a validation error based on the max-count of definitions allowed for an individual named object. Does/should skos:definition (which this field is mapped to for the purposes of vocabulary mappings) replace kgmeta:Description in this case? There’s strong validation on the kgmeta-field, perhaps there should also be a similar constraint set for equivalent skos-predicates. We probably don’t want multiple definitions for the same term.</t>
   </si>
 </sst>
 </file>
@@ -371,7 +377,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="7">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -402,13 +408,6 @@
     </font>
     <font>
       <sz val="12"/>
-      <name val="Arial"/>
-      <family val="2"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF0000FF"/>
       <name val="Arial"/>
       <family val="2"/>
       <charset val="1"/>
@@ -481,7 +480,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -519,10 +518,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -709,7 +704,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:S32"/>
+  <dimension ref="A1:S33"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="22.86"/>
@@ -1202,7 +1197,7 @@
       <c r="L17" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="S17" s="10" t="s">
+      <c r="S17" s="9" t="s">
         <v>74</v>
       </c>
     </row>
@@ -1482,7 +1477,7 @@
       <c r="I28" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="S28" s="10" t="s">
+      <c r="S28" s="9" t="s">
         <v>106</v>
       </c>
     </row>
@@ -1525,7 +1520,7 @@
       <c r="I30" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="S30" s="10" t="s">
+      <c r="S30" s="9" t="s">
         <v>109</v>
       </c>
     </row>
@@ -1548,7 +1543,7 @@
       <c r="I31" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="S31" s="10" t="s">
+      <c r="S31" s="9" t="s">
         <v>111</v>
       </c>
     </row>
@@ -1571,8 +1566,28 @@
       <c r="I32" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="S32" s="10" t="s">
+      <c r="S32" s="9" t="s">
         <v>113</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D33" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="F33" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="I33" s="2" t="s">
+        <v>115</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
incorporating visualisation functions into core
</commit_message>
<xml_diff>
--- a/tests/data/alphabet_vocab.xlsx
+++ b/tests/data/alphabet_vocab.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="266" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="267" uniqueCount="118">
   <si>
     <t xml:space="preserve">ConceptScheme</t>
   </si>
@@ -163,67 +163,73 @@
     <t xml:space="preserve">A house is a residential building typically split into different functional rooms. Houses can be built from a variety of materials and traditional houses will often reflect materials that are available locally.</t>
   </si>
   <si>
+    <t xml:space="preserve">Structure, Artifact</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://en.wikipedia.org/wiki/House</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Imagination</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Imagination is a creative cognitive process in which theories and ideas can be generated, simulated and mentally experienced.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://en.wikipedia.org/wiki/Imagination</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jungle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A jungle is a biome consisting of dense forest and tangled vegetation found in tropical climates that feature warm and humid conditions.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://en.wikipedia.org/wiki/Jungle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">King</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kaiser,Konig</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A King is a royal title given to a male monarch who rules over a nation. A realm or nation over which a monarch reigns is called a Kingdom.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Monarch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Queen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://en.wikipedia.org/wiki/King</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lemon</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A lemon is the pointed oval yellow fruit of small evergreen trees of the genus Citrus.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://en.wikipedia.org/wiki/Lemon</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mouse</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A mouse is a small rodent of the genus Mus. Mice typically have pointed snouts, small rounded ears and a long scaly tail. They can be found in multiple environments across the world, including urban environments where they can be considered vermin.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://en.wikipedia.org/wiki/Mouse</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nest</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A nest is a structure constructed by an animal to hold its eggs or young. Nests are typically attributed to birds, but members of all classes of vertebrates and some invertebrates construct nests.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Structure</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://en.wikipedia.org/wiki/House</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Imagination</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Imagination is a creative cognitive process in which theories and ideas can be generated, simulated and mentally experienced.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://en.wikipedia.org/wiki/Imagination</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jungle</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A jungle is a biome consisting of dense forest and tangled vegetation found in tropical climates that feature warm and humid conditions.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://en.wikipedia.org/wiki/Jungle</t>
-  </si>
-  <si>
-    <t xml:space="preserve">King</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A King is a royal title given to a male monarch who rules over a nation. A realm or nation over which a monarch reigns is called a Kingdom.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Monarch</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Queen</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://en.wikipedia.org/wiki/King</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lemon</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A lemon is the pointed oval yellow fruit of small evergreen trees of the genus Citrus.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://en.wikipedia.org/wiki/Lemon</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mouse</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A mouse is a small rodent of the genus Mus. Mice typically have pointed snouts, small rounded ears and a long scaly tail. They can be found in multiple environments across the world, including urban environments where they can be considered vermin.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://en.wikipedia.org/wiki/Mouse</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nest</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A nest is a structure constructed by an animal to hold its eggs or young. Nests are typically attributed to birds, but members of all classes of vertebrates and some invertebrates construct nests.</t>
   </si>
   <si>
     <t xml:space="preserve">https://en.wikipedia.org/wiki/Nest</t>
@@ -1055,20 +1061,23 @@
       <c r="F12" s="1" t="s">
         <v>55</v>
       </c>
+      <c r="G12" s="1" t="s">
+        <v>56</v>
+      </c>
       <c r="I12" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="L12" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="M12" s="1" t="s">
         <v>19</v>
       </c>
       <c r="N12" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="S12" s="9" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1082,19 +1091,19 @@
         <v>21</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="L13" s="1" t="s">
         <v>24</v>
       </c>
       <c r="S13" s="9" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1108,19 +1117,19 @@
         <v>21</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="L14" s="1" t="s">
         <v>31</v>
       </c>
       <c r="S14" s="9" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1134,19 +1143,19 @@
         <v>21</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="I15" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="L15" s="1" t="s">
-        <v>47</v>
+        <v>69</v>
       </c>
       <c r="S15" s="9" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1160,19 +1169,19 @@
         <v>21</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="I16" s="2" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="L16" s="1" t="s">
         <v>31</v>
       </c>
       <c r="S16" s="9" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1186,19 +1195,19 @@
         <v>21</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="I17" s="2" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="L17" s="1" t="s">
         <v>31</v>
       </c>
       <c r="S17" s="9" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1212,16 +1221,16 @@
         <v>21</v>
       </c>
       <c r="D18" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="F18" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="I18" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="L18" s="1" t="s">
         <v>58</v>
-      </c>
-      <c r="F18" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="I18" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="L18" s="1" t="s">
-        <v>57</v>
       </c>
       <c r="M18" s="1" t="s">
         <v>19</v>
@@ -1230,7 +1239,7 @@
         <v>55</v>
       </c>
       <c r="S18" s="9" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1244,16 +1253,16 @@
         <v>21</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="I19" s="2" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="S19" s="9" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1267,16 +1276,16 @@
         <v>21</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="I20" s="2" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="S20" s="9" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1290,19 +1299,19 @@
         <v>21</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="I21" s="2" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="L21" s="1" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="S21" s="9" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1316,19 +1325,19 @@
         <v>21</v>
       </c>
       <c r="D22" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="F22" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="I22" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="L22" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="F22" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="I22" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="L22" s="1" t="s">
-        <v>85</v>
-      </c>
       <c r="S22" s="9" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1342,16 +1351,16 @@
         <v>21</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="I23" s="2" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="S23" s="9" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1365,19 +1374,19 @@
         <v>21</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I24" s="2" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="L24" s="1" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="S24" s="9" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1391,19 +1400,19 @@
         <v>21</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="I25" s="2" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="L25" s="1" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="S25" s="9" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1417,19 +1426,19 @@
         <v>21</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="I26" s="2" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="L26" s="1" t="s">
         <v>31</v>
       </c>
       <c r="S26" s="9" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1443,19 +1452,19 @@
         <v>21</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="I27" s="2" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="L27" s="1" t="s">
         <v>31</v>
       </c>
       <c r="S27" s="9" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1475,10 +1484,10 @@
         <v>31</v>
       </c>
       <c r="I28" s="2" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="S28" s="9" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1492,13 +1501,13 @@
         <v>21</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="F29" s="1" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="I29" s="2" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1518,10 +1527,10 @@
         <v>24</v>
       </c>
       <c r="I30" s="2" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="S30" s="9" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1535,16 +1544,16 @@
         <v>21</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="F31" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="I31" s="2" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="S31" s="9" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1558,21 +1567,21 @@
         <v>21</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>47</v>
+        <v>69</v>
       </c>
       <c r="F32" s="1" t="s">
-        <v>47</v>
+        <v>69</v>
       </c>
       <c r="I32" s="2" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="S32" s="9" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="1" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="B33" s="1" t="s">
         <v>20</v>
@@ -1587,7 +1596,7 @@
         <v>22</v>
       </c>
       <c r="I33" s="2" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
     </row>
   </sheetData>

</xml_diff>